<commit_message>
tracker: dashboard sheet recalculates live from the Actions sheet
Every tile and table cell is now SUMPRODUCT(COUNTIFS(...)) over the Actions
columns (open statuses as an array constant, due dates against TODAY()), so a
status or priority changed in Excel moves the dashboard and both charts at
once. The owner and project lists are still written from the rows and refresh
on the next run. fullCalcOnLoad is set because openpyxl writes no cached
values; GitHub's file preview therefore shows the formula cells blank.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WioBNtYg1KWEYtRgYJuMkn
</commit_message>
<xml_diff>
--- a/tracker/actions.xlsx
+++ b/tracker/actions.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,12 +60,6 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="001F3864"/>
-      <sz val="22"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00C0262A"/>
       <sz val="22"/>
     </font>
     <font>
@@ -149,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -157,22 +151,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -181,13 +178,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -206,7 +203,15 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="11">
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="00C0262A"/>
+        <sz val="22"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <name val="Arial"/>
@@ -1030,7 +1035,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Snapshot generated 2026-09-17. Regenerated on every run from the Actions sheet; edit items in the Google Sheet, not here.</t>
+          <t>Live: every number is a formula over the Actions sheet, so a status changed there moves this page at once. Owner and project lists refresh on each run (last 2026-09-17). Edits that should stick belong in the Google Sheet.</t>
         </is>
       </c>
     </row>
@@ -1040,12 +1045,12 @@
           <t>OPEN ITEMS</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>P1 OPEN</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>OVERDUE</t>
         </is>
@@ -1072,30 +1077,37 @@
       </c>
     </row>
     <row r="5" ht="34" customHeight="1">
-      <c r="B5" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>17</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>3</v>
+      <c r="B5" s="5">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"}))</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$C$2:$C$5000,"P1"))</f>
+        <v/>
+      </c>
+      <c r="D5" s="6">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$E$2:$E$5000,"&lt;"&amp;TODAY()))</f>
+        <v/>
+      </c>
+      <c r="E5" s="5">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$E$2:$E$5000,TODAY()))</f>
+        <v/>
+      </c>
+      <c r="F5" s="5">
+        <f>COUNTIF(Actions!$D$2:$D$5000,"to_verify")</f>
+        <v/>
+      </c>
+      <c r="G5" s="5">
+        <f>COUNTIF(Actions!$D$2:$D$5000,"blocked")</f>
+        <v/>
+      </c>
+      <c r="H5" s="5">
+        <f>COUNTIF(Actions!$D$2:$D$5000,"done")</f>
+        <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Open items by owner</t>
         </is>
@@ -1107,193 +1119,228 @@
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
         <is>
           <t>Overdue</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Ashwini</t>
         </is>
       </c>
-      <c r="C10" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="D10" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="G10" s="10" t="n">
-        <v>3</v>
+      <c r="C10" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B10,Actions!$C$2:$C$5000,"P1"))</f>
+        <v/>
+      </c>
+      <c r="D10" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B10,Actions!$C$2:$C$5000,"P2"))</f>
+        <v/>
+      </c>
+      <c r="E10" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B10,Actions!$C$2:$C$5000,"P3"))</f>
+        <v/>
+      </c>
+      <c r="F10" s="12">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B10))</f>
+        <v/>
+      </c>
+      <c r="G10" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B10,Actions!$E$2:$E$5000,"&lt;"&amp;TODAY()))</f>
+        <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Laxmikant</t>
         </is>
       </c>
-      <c r="C11" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="D11" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="G11" s="10" t="n">
-        <v>4</v>
+      <c r="C11" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B11,Actions!$C$2:$C$5000,"P1"))</f>
+        <v/>
+      </c>
+      <c r="D11" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B11,Actions!$C$2:$C$5000,"P2"))</f>
+        <v/>
+      </c>
+      <c r="E11" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B11,Actions!$C$2:$C$5000,"P3"))</f>
+        <v/>
+      </c>
+      <c r="F11" s="12">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B11))</f>
+        <v/>
+      </c>
+      <c r="G11" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B11,Actions!$E$2:$E$5000,"&lt;"&amp;TODAY()))</f>
+        <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Johan</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D12" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="G12" s="10" t="n">
-        <v>4</v>
+      <c r="C12" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B12,Actions!$C$2:$C$5000,"P1"))</f>
+        <v/>
+      </c>
+      <c r="D12" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B12,Actions!$C$2:$C$5000,"P2"))</f>
+        <v/>
+      </c>
+      <c r="E12" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B12,Actions!$C$2:$C$5000,"P3"))</f>
+        <v/>
+      </c>
+      <c r="F12" s="12">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B12))</f>
+        <v/>
+      </c>
+      <c r="G12" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B12,Actions!$E$2:$E$5000,"&lt;"&amp;TODAY()))</f>
+        <v/>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Samuel</t>
         </is>
       </c>
-      <c r="C13" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D13" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="G13" s="10" t="n">
-        <v>4</v>
+      <c r="C13" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B13,Actions!$C$2:$C$5000,"P1"))</f>
+        <v/>
+      </c>
+      <c r="D13" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B13,Actions!$C$2:$C$5000,"P2"))</f>
+        <v/>
+      </c>
+      <c r="E13" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B13,Actions!$C$2:$C$5000,"P3"))</f>
+        <v/>
+      </c>
+      <c r="F13" s="12">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B13))</f>
+        <v/>
+      </c>
+      <c r="G13" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B13,Actions!$E$2:$E$5000,"&lt;"&amp;TODAY()))</f>
+        <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Ayush</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G14" s="10" t="n">
-        <v>2</v>
+      <c r="C14" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B14,Actions!$C$2:$C$5000,"P1"))</f>
+        <v/>
+      </c>
+      <c r="D14" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B14,Actions!$C$2:$C$5000,"P2"))</f>
+        <v/>
+      </c>
+      <c r="E14" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B14,Actions!$C$2:$C$5000,"P3"))</f>
+        <v/>
+      </c>
+      <c r="F14" s="12">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B14))</f>
+        <v/>
+      </c>
+      <c r="G14" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B14,Actions!$E$2:$E$5000,"&lt;"&amp;TODAY()))</f>
+        <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Sarathchandra Babu</t>
         </is>
       </c>
-      <c r="C15" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="10" t="n">
-        <v>0</v>
+      <c r="C15" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B15,Actions!$C$2:$C$5000,"P1"))</f>
+        <v/>
+      </c>
+      <c r="D15" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B15,Actions!$C$2:$C$5000,"P2"))</f>
+        <v/>
+      </c>
+      <c r="E15" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B15,Actions!$C$2:$C$5000,"P3"))</f>
+        <v/>
+      </c>
+      <c r="F15" s="12">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B15))</f>
+        <v/>
+      </c>
+      <c r="G15" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$B$2:$B$5000,$B15,Actions!$E$2:$E$5000,"&lt;"&amp;TODAY()))</f>
+        <v/>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C16" s="13" t="n">
-        <v>14</v>
-      </c>
-      <c r="D16" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="E16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="13" t="n">
-        <v>19</v>
-      </c>
-      <c r="G16" s="13" t="n">
-        <v>17</v>
+      <c r="C16" s="14">
+        <f>SUM(C10:C15)</f>
+        <v/>
+      </c>
+      <c r="D16" s="14">
+        <f>SUM(D10:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="14">
+        <f>SUM(E10:E15)</f>
+        <v/>
+      </c>
+      <c r="F16" s="14">
+        <f>SUM(F10:F15)</f>
+        <v/>
+      </c>
+      <c r="G16" s="14">
+        <f>SUM(G10:G15)</f>
+        <v/>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>When is it due</t>
         </is>
@@ -1305,255 +1352,283 @@
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Horizon</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>Items</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>Overdue</t>
         </is>
       </c>
-      <c r="C24" s="11" t="n">
-        <v>17</v>
-      </c>
-      <c r="D24" s="10" t="n">
-        <v>13</v>
+      <c r="C24" s="12">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$E$2:$E$5000,"&lt;"&amp;TODAY()))</f>
+        <v/>
+      </c>
+      <c r="D24" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$E$2:$E$5000,"&lt;"&amp;TODAY(),Actions!$C$2:$C$5000,"P1"))</f>
+        <v/>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>Due today</t>
         </is>
       </c>
-      <c r="C25" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="10" t="n">
-        <v>0</v>
+      <c r="C25" s="12">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$E$2:$E$5000,TODAY()))</f>
+        <v/>
+      </c>
+      <c r="D25" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$E$2:$E$5000,TODAY(),Actions!$C$2:$C$5000,"P1"))</f>
+        <v/>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>Next 7 days</t>
         </is>
       </c>
-      <c r="C26" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="10" t="n">
-        <v>0</v>
+      <c r="C26" s="12">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$E$2:$E$5000,"&gt;"&amp;TODAY(),Actions!$E$2:$E$5000,"&lt;="&amp;TODAY()+7))</f>
+        <v/>
+      </c>
+      <c r="D26" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$E$2:$E$5000,"&gt;"&amp;TODAY(),Actions!$E$2:$E$5000,"&lt;="&amp;TODAY()+7,Actions!$C$2:$C$5000,"P1"))</f>
+        <v/>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>Later</t>
         </is>
       </c>
-      <c r="C27" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="10" t="n">
-        <v>0</v>
+      <c r="C27" s="12">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$E$2:$E$5000,"&gt;"&amp;TODAY()+7))</f>
+        <v/>
+      </c>
+      <c r="D27" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$E$2:$E$5000,"&gt;"&amp;TODAY()+7,Actions!$C$2:$C$5000,"P1"))</f>
+        <v/>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>No date</t>
         </is>
       </c>
-      <c r="C28" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="10" t="n">
-        <v>1</v>
+      <c r="C28" s="12">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$E$2:$E$5000,""))</f>
+        <v/>
+      </c>
+      <c r="D28" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$E$2:$E$5000,"",Actions!$C$2:$C$5000,"P1"))</f>
+        <v/>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>By project</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="D32" s="8" t="inlineStr">
+      <c r="D32" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E32" s="8" t="inlineStr">
+      <c r="E32" s="9" t="inlineStr">
         <is>
           <t>Overdue</t>
         </is>
       </c>
-      <c r="F32" s="8" t="inlineStr">
+      <c r="F32" s="9" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="C33" s="11" t="n">
-        <v>18</v>
-      </c>
-      <c r="D33" s="10" t="n">
-        <v>14</v>
-      </c>
-      <c r="E33" s="10" t="n">
-        <v>17</v>
-      </c>
-      <c r="F33" s="10" t="n">
-        <v>0</v>
+      <c r="C33" s="12">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$F$2:$F$5000,$B33))</f>
+        <v/>
+      </c>
+      <c r="D33" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$F$2:$F$5000,$B33,Actions!$C$2:$C$5000,"P1"))</f>
+        <v/>
+      </c>
+      <c r="E33" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$F$2:$F$5000,$B33,Actions!$E$2:$E$5000,"&lt;"&amp;TODAY()))</f>
+        <v/>
+      </c>
+      <c r="F33" s="11">
+        <f>COUNTIFS(Actions!$F$2:$F$5000,$B33,Actions!$D$2:$D$5000,"done")</f>
+        <v/>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>lsp</t>
         </is>
       </c>
-      <c r="C34" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" s="10" t="n">
-        <v>3</v>
+      <c r="C34" s="12">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$F$2:$F$5000,$B34))</f>
+        <v/>
+      </c>
+      <c r="D34" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$F$2:$F$5000,$B34,Actions!$C$2:$C$5000,"P1"))</f>
+        <v/>
+      </c>
+      <c r="E34" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$F$2:$F$5000,$B34,Actions!$E$2:$E$5000,"&lt;"&amp;TODAY()))</f>
+        <v/>
+      </c>
+      <c r="F34" s="11">
+        <f>COUNTIFS(Actions!$F$2:$F$5000,$B34,Actions!$D$2:$D$5000,"done")</f>
+        <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>unassigned</t>
         </is>
       </c>
-      <c r="C35" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="10" t="n">
-        <v>0</v>
+      <c r="C35" s="12">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$F$2:$F$5000,$B35))</f>
+        <v/>
+      </c>
+      <c r="D35" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$F$2:$F$5000,$B35,Actions!$C$2:$C$5000,"P1"))</f>
+        <v/>
+      </c>
+      <c r="E35" s="11">
+        <f>SUMPRODUCT(COUNTIFS(Actions!$D$2:$D$5000,{"blocked","in_progress","open","to_verify"},Actions!$F$2:$F$5000,$B35,Actions!$E$2:$E$5000,"&lt;"&amp;TODAY()))</f>
+        <v/>
+      </c>
+      <c r="F35" s="11">
+        <f>COUNTIFS(Actions!$F$2:$F$5000,$B35,Actions!$D$2:$D$5000,"done")</f>
+        <v/>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="6" t="inlineStr">
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>By status</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="B39" s="7" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C39" s="8" t="inlineStr">
+      <c r="C39" s="9" t="inlineStr">
         <is>
           <t>Items</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="9" t="inlineStr">
+      <c r="B40" s="10" t="inlineStr">
         <is>
           <t>blocked</t>
         </is>
       </c>
-      <c r="C40" s="11" t="n">
-        <v>0</v>
+      <c r="C40" s="12">
+        <f>COUNTIF(Actions!$D$2:$D$5000,$B40)</f>
+        <v/>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="9" t="inlineStr">
+      <c r="B41" s="10" t="inlineStr">
         <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="C41" s="11" t="n">
-        <v>1</v>
+      <c r="C41" s="12">
+        <f>COUNTIF(Actions!$D$2:$D$5000,$B41)</f>
+        <v/>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="9" t="inlineStr">
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="C42" s="11" t="n">
-        <v>18</v>
+      <c r="C42" s="12">
+        <f>COUNTIF(Actions!$D$2:$D$5000,$B42)</f>
+        <v/>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="9" t="inlineStr">
+      <c r="B43" s="10" t="inlineStr">
         <is>
           <t>to_verify</t>
         </is>
       </c>
-      <c r="C43" s="11" t="n">
-        <v>0</v>
+      <c r="C43" s="12">
+        <f>COUNTIF(Actions!$D$2:$D$5000,$B43)</f>
+        <v/>
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="9" t="inlineStr">
+      <c r="B44" s="10" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="C44" s="11" t="n">
-        <v>3</v>
+      <c r="C44" s="12">
+        <f>COUNTIF(Actions!$D$2:$D$5000,$B44)</f>
+        <v/>
       </c>
     </row>
     <row r="45">
-      <c r="B45" s="9" t="inlineStr">
+      <c r="B45" s="10" t="inlineStr">
         <is>
           <t>rejected</t>
         </is>
       </c>
-      <c r="C45" s="11" t="n">
-        <v>0</v>
+      <c r="C45" s="12">
+        <f>COUNTIF(Actions!$D$2:$D$5000,$B45)</f>
+        <v/>
       </c>
     </row>
     <row r="47" ht="16" customHeight="1">
@@ -1571,6 +1646,16 @@
     <mergeCell ref="B47:Q48"/>
     <mergeCell ref="D22:Q22"/>
   </mergeCells>
+  <conditionalFormatting sqref="C5">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>C5&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D5">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>D5&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -1611,1837 +1696,1837 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>task</t>
         </is>
       </c>
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>owner</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
         <is>
           <t>priority</t>
         </is>
       </c>
-      <c r="D1" s="14" t="inlineStr">
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="E1" s="14" t="inlineStr">
+      <c r="E1" s="15" t="inlineStr">
         <is>
           <t>due</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
+      <c r="F1" s="15" t="inlineStr">
         <is>
           <t>project</t>
         </is>
       </c>
-      <c r="G1" s="14" t="inlineStr">
+      <c r="G1" s="15" t="inlineStr">
         <is>
           <t>team</t>
         </is>
       </c>
-      <c r="H1" s="14" t="inlineStr">
+      <c r="H1" s="15" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="I1" s="14" t="inlineStr">
+      <c r="I1" s="15" t="inlineStr">
         <is>
           <t>next_step</t>
         </is>
       </c>
-      <c r="J1" s="14" t="inlineStr">
+      <c r="J1" s="15" t="inlineStr">
         <is>
           <t>unblocker</t>
         </is>
       </c>
-      <c r="K1" s="14" t="inlineStr">
+      <c r="K1" s="15" t="inlineStr">
         <is>
           <t>effort</t>
         </is>
       </c>
-      <c r="L1" s="14" t="inlineStr">
+      <c r="L1" s="15" t="inlineStr">
         <is>
           <t>blocked_by</t>
         </is>
       </c>
-      <c r="M1" s="14" t="inlineStr">
+      <c r="M1" s="15" t="inlineStr">
         <is>
           <t>prerequisites</t>
         </is>
       </c>
-      <c r="N1" s="14" t="inlineStr">
+      <c r="N1" s="15" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="O1" s="14" t="inlineStr">
+      <c r="O1" s="15" t="inlineStr">
         <is>
           <t>evidence</t>
         </is>
       </c>
-      <c r="P1" s="14" t="inlineStr">
+      <c r="P1" s="15" t="inlineStr">
         <is>
           <t>basis</t>
         </is>
       </c>
-      <c r="Q1" s="14" t="inlineStr">
+      <c r="Q1" s="15" t="inlineStr">
         <is>
           <t>meeting</t>
         </is>
       </c>
-      <c r="R1" s="14" t="inlineStr">
+      <c r="R1" s="15" t="inlineStr">
         <is>
           <t>origin</t>
         </is>
       </c>
-      <c r="S1" s="14" t="inlineStr">
+      <c r="S1" s="15" t="inlineStr">
         <is>
           <t>updated</t>
         </is>
       </c>
-      <c r="T1" s="14" t="inlineStr">
+      <c r="T1" s="15" t="inlineStr">
         <is>
           <t>closed</t>
         </is>
       </c>
-      <c r="U1" s="14" t="inlineStr">
+      <c r="U1" s="15" t="inlineStr">
         <is>
           <t>created</t>
         </is>
       </c>
-      <c r="V1" s="14" t="inlineStr">
+      <c r="V1" s="15" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="W1" s="14" t="inlineStr">
+      <c r="W1" s="15" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Sign off on the reviewed database design after today's walkthrough.</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="B2" s="16" t="inlineStr">
         <is>
           <t>Ashwini</t>
         </is>
       </c>
-      <c r="C2" s="16" t="inlineStr">
+      <c r="C2" s="17" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D2" s="16" t="inlineStr">
+      <c r="D2" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E2" s="17" t="n">
+      <c r="E2" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="F2" s="15" t="inlineStr">
+      <c r="F2" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G2" s="15" t="inlineStr">
+      <c r="G2" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H2" s="15" t="inlineStr"/>
-      <c r="I2" s="15" t="inlineStr"/>
-      <c r="J2" s="15" t="inlineStr"/>
-      <c r="K2" s="16" t="inlineStr"/>
-      <c r="L2" s="15" t="inlineStr"/>
-      <c r="M2" s="15" t="inlineStr"/>
-      <c r="N2" s="15" t="inlineStr"/>
-      <c r="O2" s="15" t="inlineStr">
+      <c r="H2" s="16" t="inlineStr"/>
+      <c r="I2" s="16" t="inlineStr"/>
+      <c r="J2" s="16" t="inlineStr"/>
+      <c r="K2" s="17" t="inlineStr"/>
+      <c r="L2" s="16" t="inlineStr"/>
+      <c r="M2" s="16" t="inlineStr"/>
+      <c r="N2" s="16" t="inlineStr"/>
+      <c r="O2" s="16" t="inlineStr">
         <is>
           <t>I will be signing off on the Debi after the review</t>
         </is>
       </c>
-      <c r="P2" s="15" t="inlineStr"/>
-      <c r="Q2" s="15" t="inlineStr">
+      <c r="P2" s="16" t="inlineStr"/>
+      <c r="Q2" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R2" s="16" t="inlineStr">
+      <c r="R2" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S2" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T2" s="17" t="n"/>
-      <c r="U2" s="17" t="n">
+      <c r="S2" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T2" s="18" t="n"/>
+      <c r="U2" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="V2" s="15" t="inlineStr">
+      <c r="V2" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W2" s="15" t="inlineStr">
+      <c r="W2" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-intelligent-tracker-01</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Work with Ashwini on the overall workflow solution design document.</t>
         </is>
       </c>
-      <c r="B3" s="15" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>Laxmikant</t>
         </is>
       </c>
-      <c r="C3" s="16" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D3" s="16" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E3" s="17" t="n">
+      <c r="E3" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="F3" s="15" t="inlineStr">
+      <c r="F3" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G3" s="15" t="inlineStr">
+      <c r="G3" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H3" s="15" t="inlineStr"/>
-      <c r="I3" s="15" t="inlineStr"/>
-      <c r="J3" s="15" t="inlineStr"/>
-      <c r="K3" s="16" t="inlineStr"/>
-      <c r="L3" s="15" t="inlineStr"/>
-      <c r="M3" s="15" t="inlineStr"/>
-      <c r="N3" s="15" t="inlineStr"/>
-      <c r="O3" s="15" t="inlineStr">
+      <c r="H3" s="16" t="inlineStr"/>
+      <c r="I3" s="16" t="inlineStr"/>
+      <c r="J3" s="16" t="inlineStr"/>
+      <c r="K3" s="17" t="inlineStr"/>
+      <c r="L3" s="16" t="inlineStr"/>
+      <c r="M3" s="16" t="inlineStr"/>
+      <c r="N3" s="16" t="inlineStr"/>
+      <c r="O3" s="16" t="inlineStr">
         <is>
           <t>Lakshmi and I will be working on the proper workflow solution design</t>
         </is>
       </c>
-      <c r="P3" s="15" t="inlineStr"/>
-      <c r="Q3" s="15" t="inlineStr">
+      <c r="P3" s="16" t="inlineStr"/>
+      <c r="Q3" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R3" s="16" t="inlineStr">
+      <c r="R3" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S3" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T3" s="17" t="n"/>
-      <c r="U3" s="17" t="n">
+      <c r="S3" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T3" s="18" t="n"/>
+      <c r="U3" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="V3" s="15" t="inlineStr">
+      <c r="V3" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W3" s="15" t="inlineStr">
+      <c r="W3" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-intelligent-tracker-04</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Change the CR Notes field UI from a single-line text box to a multi-line text box as Sreekumar requested.</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>Johan</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E4" s="17" t="n">
+      <c r="E4" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="F4" s="15" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G4" s="15" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H4" s="15" t="inlineStr"/>
-      <c r="I4" s="15" t="inlineStr"/>
-      <c r="J4" s="15" t="inlineStr"/>
-      <c r="K4" s="16" t="inlineStr"/>
-      <c r="L4" s="15" t="inlineStr"/>
-      <c r="M4" s="15" t="inlineStr"/>
-      <c r="N4" s="15" t="inlineStr"/>
-      <c r="O4" s="15" t="inlineStr">
+      <c r="H4" s="16" t="inlineStr"/>
+      <c r="I4" s="16" t="inlineStr"/>
+      <c r="J4" s="16" t="inlineStr"/>
+      <c r="K4" s="17" t="inlineStr"/>
+      <c r="L4" s="16" t="inlineStr"/>
+      <c r="M4" s="16" t="inlineStr"/>
+      <c r="N4" s="16" t="inlineStr"/>
+      <c r="O4" s="16" t="inlineStr">
         <is>
           <t>Change the UI. I'll change it.</t>
         </is>
       </c>
-      <c r="P4" s="15" t="inlineStr"/>
-      <c r="Q4" s="15" t="inlineStr">
+      <c r="P4" s="16" t="inlineStr"/>
+      <c r="Q4" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R4" s="16" t="inlineStr">
+      <c r="R4" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S4" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T4" s="17" t="n"/>
-      <c r="U4" s="17" t="n">
+      <c r="S4" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T4" s="18" t="n"/>
+      <c r="U4" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="V4" s="15" t="inlineStr">
+      <c r="V4" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W4" s="15" t="inlineStr">
+      <c r="W4" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-intelligent-tracker-05</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Write detailed user stories for the Change Request module workflow and share them with Ashwini and Laxmikant.</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Johan</t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E5" s="17" t="n">
+      <c r="E5" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="F5" s="15" t="inlineStr">
+      <c r="F5" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G5" s="15" t="inlineStr">
+      <c r="G5" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H5" s="15" t="inlineStr"/>
-      <c r="I5" s="15" t="inlineStr"/>
-      <c r="J5" s="15" t="inlineStr"/>
-      <c r="K5" s="16" t="inlineStr"/>
-      <c r="L5" s="15" t="inlineStr"/>
-      <c r="M5" s="15" t="inlineStr"/>
-      <c r="N5" s="15" t="inlineStr"/>
-      <c r="O5" s="15" t="inlineStr">
+      <c r="H5" s="16" t="inlineStr"/>
+      <c r="I5" s="16" t="inlineStr"/>
+      <c r="J5" s="16" t="inlineStr"/>
+      <c r="K5" s="17" t="inlineStr"/>
+      <c r="L5" s="16" t="inlineStr"/>
+      <c r="M5" s="16" t="inlineStr"/>
+      <c r="N5" s="16" t="inlineStr"/>
+      <c r="O5" s="16" t="inlineStr">
         <is>
           <t>you share it to Ashwini B and Lakshmi Lakshmi</t>
         </is>
       </c>
-      <c r="P5" s="15" t="inlineStr"/>
-      <c r="Q5" s="15" t="inlineStr">
+      <c r="P5" s="16" t="inlineStr"/>
+      <c r="Q5" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R5" s="16" t="inlineStr">
+      <c r="R5" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S5" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T5" s="17" t="n"/>
-      <c r="U5" s="17" t="n">
+      <c r="S5" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T5" s="18" t="n"/>
+      <c r="U5" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="V5" s="15" t="inlineStr">
+      <c r="V5" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W5" s="15" t="inlineStr">
+      <c r="W5" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-intelligent-tracker-06</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>Write detailed user stories for the Issues module workflow and present them to Ayush.</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>Samuel</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E6" s="17" t="n">
+      <c r="E6" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="F6" s="15" t="inlineStr">
+      <c r="F6" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G6" s="15" t="inlineStr">
+      <c r="G6" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H6" s="15" t="inlineStr"/>
-      <c r="I6" s="15" t="inlineStr"/>
-      <c r="J6" s="15" t="inlineStr"/>
-      <c r="K6" s="16" t="inlineStr"/>
-      <c r="L6" s="15" t="inlineStr"/>
-      <c r="M6" s="15" t="inlineStr"/>
-      <c r="N6" s="15" t="inlineStr"/>
-      <c r="O6" s="15" t="inlineStr">
+      <c r="H6" s="16" t="inlineStr"/>
+      <c r="I6" s="16" t="inlineStr"/>
+      <c r="J6" s="16" t="inlineStr"/>
+      <c r="K6" s="17" t="inlineStr"/>
+      <c r="L6" s="16" t="inlineStr"/>
+      <c r="M6" s="16" t="inlineStr"/>
+      <c r="N6" s="16" t="inlineStr"/>
+      <c r="O6" s="16" t="inlineStr">
         <is>
           <t>user stories you figure out and you show me</t>
         </is>
       </c>
-      <c r="P6" s="15" t="inlineStr"/>
-      <c r="Q6" s="15" t="inlineStr">
+      <c r="P6" s="16" t="inlineStr"/>
+      <c r="Q6" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R6" s="16" t="inlineStr">
+      <c r="R6" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S6" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T6" s="17" t="n"/>
-      <c r="U6" s="17" t="n">
+      <c r="S6" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T6" s="18" t="n"/>
+      <c r="U6" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="V6" s="15" t="inlineStr">
+      <c r="V6" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W6" s="15" t="inlineStr">
+      <c r="W6" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-intelligent-tracker-07</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Complete the SharePoint list configuration for the DB changes made last Friday and update the UI design to match.</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>Laxmikant</t>
         </is>
       </c>
-      <c r="C7" s="16" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="E7" s="18" t="n">
         <v>46280</v>
       </c>
-      <c r="F7" s="15" t="inlineStr">
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G7" s="15" t="inlineStr">
+      <c r="G7" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H7" s="15" t="inlineStr"/>
-      <c r="I7" s="15" t="inlineStr"/>
-      <c r="J7" s="15" t="inlineStr"/>
-      <c r="K7" s="16" t="inlineStr"/>
-      <c r="L7" s="15" t="inlineStr"/>
-      <c r="M7" s="15" t="inlineStr"/>
-      <c r="N7" s="15" t="inlineStr"/>
-      <c r="O7" s="15" t="inlineStr">
+      <c r="H7" s="16" t="inlineStr"/>
+      <c r="I7" s="16" t="inlineStr"/>
+      <c r="J7" s="16" t="inlineStr"/>
+      <c r="K7" s="17" t="inlineStr"/>
+      <c r="L7" s="16" t="inlineStr"/>
+      <c r="M7" s="16" t="inlineStr"/>
+      <c r="N7" s="16" t="inlineStr"/>
+      <c r="O7" s="16" t="inlineStr">
         <is>
           <t>Lakshmi will be doing the SharePoint configuration, whatever related to DB changes last Friday we did.</t>
         </is>
       </c>
-      <c r="P7" s="15" t="inlineStr"/>
-      <c r="Q7" s="15" t="inlineStr">
+      <c r="P7" s="16" t="inlineStr"/>
+      <c r="Q7" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R7" s="16" t="inlineStr">
+      <c r="R7" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S7" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T7" s="17" t="n"/>
-      <c r="U7" s="17" t="n">
+      <c r="S7" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T7" s="18" t="n"/>
+      <c r="U7" s="18" t="n">
         <v>46280</v>
       </c>
-      <c r="V7" s="15" t="inlineStr">
+      <c r="V7" s="16" t="inlineStr">
         <is>
           <t>2026-09-15-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W7" s="15" t="inlineStr">
+      <c r="W7" s="16" t="inlineStr">
         <is>
           <t>2026-09-15-intelligent-tracker-01</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Update the Issues module UI design and start Canvas development once it is complete.</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>Samuel</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D8" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E8" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="F8" s="15" t="inlineStr">
+      <c r="E8" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G8" s="15" t="inlineStr">
+      <c r="G8" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H8" s="15" t="inlineStr"/>
-      <c r="I8" s="15" t="inlineStr"/>
-      <c r="J8" s="15" t="inlineStr"/>
-      <c r="K8" s="16" t="inlineStr"/>
-      <c r="L8" s="15" t="inlineStr"/>
-      <c r="M8" s="15" t="inlineStr"/>
-      <c r="N8" s="15" t="inlineStr">
+      <c r="H8" s="16" t="inlineStr"/>
+      <c r="I8" s="16" t="inlineStr"/>
+      <c r="J8" s="16" t="inlineStr"/>
+      <c r="K8" s="17" t="inlineStr"/>
+      <c r="L8" s="16" t="inlineStr"/>
+      <c r="M8" s="16" t="inlineStr"/>
+      <c r="N8" s="16" t="inlineStr">
         <is>
           <t>2026-09-16: Sreekumar added new review points (root cause, resolution, attachment capture, status dropdown) that must be incorporated before this task is complete; due date extended to today.</t>
         </is>
       </c>
-      <c r="O8" s="15" t="inlineStr">
+      <c r="O8" s="16" t="inlineStr">
         <is>
           <t>Samuel also, he will update the UI design. So if it is done, so he will start with the development.</t>
         </is>
       </c>
-      <c r="P8" s="15" t="inlineStr"/>
-      <c r="Q8" s="15" t="inlineStr">
+      <c r="P8" s="16" t="inlineStr"/>
+      <c r="Q8" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R8" s="16" t="inlineStr">
+      <c r="R8" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S8" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T8" s="17" t="n"/>
-      <c r="U8" s="17" t="n">
+      <c r="S8" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T8" s="18" t="n"/>
+      <c r="U8" s="18" t="n">
         <v>46280</v>
       </c>
-      <c r="V8" s="15" t="inlineStr">
+      <c r="V8" s="16" t="inlineStr">
         <is>
           <t>2026-09-15-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W8" s="15" t="inlineStr">
+      <c r="W8" s="16" t="inlineStr">
         <is>
           <t>2026-09-15-intelligent-tracker-02</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Review how developers close issues in Zoho (root cause, resolution, attachments) and identify fields to replicate in the Issues module UI.</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Ashwini</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E9" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="F9" s="15" t="inlineStr">
+      <c r="E9" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G9" s="15" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H9" s="15" t="inlineStr"/>
-      <c r="I9" s="15" t="inlineStr"/>
-      <c r="J9" s="15" t="inlineStr"/>
-      <c r="K9" s="16" t="inlineStr"/>
-      <c r="L9" s="15" t="inlineStr"/>
-      <c r="M9" s="15" t="inlineStr"/>
-      <c r="N9" s="15" t="inlineStr"/>
-      <c r="O9" s="15" t="inlineStr">
+      <c r="H9" s="16" t="inlineStr"/>
+      <c r="I9" s="16" t="inlineStr"/>
+      <c r="J9" s="16" t="inlineStr"/>
+      <c r="K9" s="17" t="inlineStr"/>
+      <c r="L9" s="16" t="inlineStr"/>
+      <c r="M9" s="16" t="inlineStr"/>
+      <c r="N9" s="16" t="inlineStr"/>
+      <c r="O9" s="16" t="inlineStr">
         <is>
           <t>Ashwini, how a developer is closing a task? Just look at that once again in Zoho.</t>
         </is>
       </c>
-      <c r="P9" s="15" t="inlineStr"/>
-      <c r="Q9" s="15" t="inlineStr">
+      <c r="P9" s="16" t="inlineStr"/>
+      <c r="Q9" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R9" s="16" t="inlineStr">
+      <c r="R9" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S9" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T9" s="17" t="n"/>
-      <c r="U9" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="V9" s="15" t="inlineStr">
+      <c r="S9" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T9" s="18" t="n"/>
+      <c r="U9" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="V9" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W9" s="15" t="inlineStr">
+      <c r="W9" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-intelligent-tracker-02</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Add the currency selector column to the CR entry screen UI (currently only present in the impact analysis view).</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>Johan</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D10" s="16" t="inlineStr">
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E10" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="F10" s="15" t="inlineStr">
+      <c r="E10" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G10" s="15" t="inlineStr">
+      <c r="G10" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H10" s="15" t="inlineStr"/>
-      <c r="I10" s="15" t="inlineStr"/>
-      <c r="J10" s="15" t="inlineStr"/>
-      <c r="K10" s="16" t="inlineStr"/>
-      <c r="L10" s="15" t="inlineStr"/>
-      <c r="M10" s="15" t="inlineStr"/>
-      <c r="N10" s="15" t="inlineStr"/>
-      <c r="O10" s="15" t="inlineStr">
+      <c r="H10" s="16" t="inlineStr"/>
+      <c r="I10" s="16" t="inlineStr"/>
+      <c r="J10" s="16" t="inlineStr"/>
+      <c r="K10" s="17" t="inlineStr"/>
+      <c r="L10" s="16" t="inlineStr"/>
+      <c r="M10" s="16" t="inlineStr"/>
+      <c r="N10" s="16" t="inlineStr"/>
+      <c r="O10" s="16" t="inlineStr">
         <is>
           <t>you'll be adding that column in that entry screen, CR entry screen. It is not there now.</t>
         </is>
       </c>
-      <c r="P10" s="15" t="inlineStr"/>
-      <c r="Q10" s="15" t="inlineStr">
+      <c r="P10" s="16" t="inlineStr"/>
+      <c r="Q10" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R10" s="16" t="inlineStr">
+      <c r="R10" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S10" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T10" s="17" t="n"/>
-      <c r="U10" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="V10" s="15" t="inlineStr">
+      <c r="S10" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T10" s="18" t="n"/>
+      <c r="U10" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="V10" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W10" s="15" t="inlineStr">
+      <c r="W10" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-intelligent-tracker-03</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>Add phase-level delay visibility (green/red per stage, payment milestone impact) and a morning alert for predicted delays to the project screen.</t>
         </is>
       </c>
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>Laxmikant</t>
         </is>
       </c>
-      <c r="C11" s="16" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E11" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="F11" s="15" t="inlineStr">
+      <c r="E11" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G11" s="15" t="inlineStr">
+      <c r="G11" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H11" s="15" t="inlineStr"/>
-      <c r="I11" s="15" t="inlineStr"/>
-      <c r="J11" s="15" t="inlineStr"/>
-      <c r="K11" s="16" t="inlineStr"/>
-      <c r="L11" s="15" t="inlineStr"/>
-      <c r="M11" s="15" t="inlineStr"/>
-      <c r="N11" s="15" t="inlineStr"/>
-      <c r="O11" s="15" t="inlineStr">
+      <c r="H11" s="16" t="inlineStr"/>
+      <c r="I11" s="16" t="inlineStr"/>
+      <c r="J11" s="16" t="inlineStr"/>
+      <c r="K11" s="17" t="inlineStr"/>
+      <c r="L11" s="16" t="inlineStr"/>
+      <c r="M11" s="16" t="inlineStr"/>
+      <c r="N11" s="16" t="inlineStr"/>
+      <c r="O11" s="16" t="inlineStr">
         <is>
           <t>Every day morning they should know that what is a predicted problem that can happen in the future.</t>
         </is>
       </c>
-      <c r="P11" s="15" t="inlineStr"/>
-      <c r="Q11" s="15" t="inlineStr">
+      <c r="P11" s="16" t="inlineStr"/>
+      <c r="Q11" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R11" s="16" t="inlineStr">
+      <c r="R11" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S11" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T11" s="17" t="n"/>
-      <c r="U11" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="V11" s="15" t="inlineStr">
+      <c r="S11" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T11" s="18" t="n"/>
+      <c r="U11" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="V11" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W11" s="15" t="inlineStr">
+      <c r="W11" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-intelligent-tracker-04</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>Add separate flags for CR effort-vs-estimate overrun and schedule slip in the time tracker.</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>Laxmikant</t>
         </is>
       </c>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="C12" s="17" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E12" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="F12" s="15" t="inlineStr">
+      <c r="E12" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G12" s="15" t="inlineStr">
+      <c r="G12" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H12" s="15" t="inlineStr"/>
-      <c r="I12" s="15" t="inlineStr"/>
-      <c r="J12" s="15" t="inlineStr"/>
-      <c r="K12" s="16" t="inlineStr"/>
-      <c r="L12" s="15" t="inlineStr"/>
-      <c r="M12" s="15" t="inlineStr"/>
-      <c r="N12" s="15" t="inlineStr"/>
-      <c r="O12" s="15" t="inlineStr">
+      <c r="H12" s="16" t="inlineStr"/>
+      <c r="I12" s="16" t="inlineStr"/>
+      <c r="J12" s="16" t="inlineStr"/>
+      <c r="K12" s="17" t="inlineStr"/>
+      <c r="L12" s="16" t="inlineStr"/>
+      <c r="M12" s="16" t="inlineStr"/>
+      <c r="N12" s="16" t="inlineStr"/>
+      <c r="O12" s="16" t="inlineStr">
         <is>
           <t>there will be definitely a flat. Yes, estimated hours versus total hours will be there, sir.</t>
         </is>
       </c>
-      <c r="P12" s="15" t="inlineStr"/>
-      <c r="Q12" s="15" t="inlineStr">
+      <c r="P12" s="16" t="inlineStr"/>
+      <c r="Q12" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R12" s="16" t="inlineStr">
+      <c r="R12" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S12" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T12" s="17" t="n"/>
-      <c r="U12" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="V12" s="15" t="inlineStr">
+      <c r="S12" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T12" s="18" t="n"/>
+      <c r="U12" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="V12" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W12" s="15" t="inlineStr">
+      <c r="W12" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-intelligent-tracker-05</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>Post today's review comments for Issues, CR and Plan Tree in the group chat so Sreekumar can give sign-off.</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>Ashwini</t>
         </is>
       </c>
-      <c r="C13" s="16" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D13" s="16" t="inlineStr">
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E13" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="F13" s="15" t="inlineStr">
+      <c r="E13" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G13" s="15" t="inlineStr">
+      <c r="G13" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H13" s="15" t="inlineStr"/>
-      <c r="I13" s="15" t="inlineStr"/>
-      <c r="J13" s="15" t="inlineStr"/>
-      <c r="K13" s="16" t="inlineStr"/>
-      <c r="L13" s="15" t="inlineStr"/>
-      <c r="M13" s="15" t="inlineStr"/>
-      <c r="N13" s="15" t="inlineStr"/>
-      <c r="O13" s="15" t="inlineStr">
+      <c r="H13" s="16" t="inlineStr"/>
+      <c r="I13" s="16" t="inlineStr"/>
+      <c r="J13" s="16" t="inlineStr"/>
+      <c r="K13" s="17" t="inlineStr"/>
+      <c r="L13" s="16" t="inlineStr"/>
+      <c r="M13" s="16" t="inlineStr"/>
+      <c r="N13" s="16" t="inlineStr"/>
+      <c r="O13" s="16" t="inlineStr">
         <is>
           <t>make sure that we put those review comments in the group. Based on that, I will give you the sign off in the chat.</t>
         </is>
       </c>
-      <c r="P13" s="15" t="inlineStr"/>
-      <c r="Q13" s="15" t="inlineStr">
+      <c r="P13" s="16" t="inlineStr"/>
+      <c r="Q13" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R13" s="16" t="inlineStr">
+      <c r="R13" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S13" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T13" s="17" t="n"/>
-      <c r="U13" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="V13" s="15" t="inlineStr">
+      <c r="S13" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T13" s="18" t="n"/>
+      <c r="U13" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="V13" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W13" s="15" t="inlineStr">
+      <c r="W13" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-intelligent-tracker-06</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Review Laxmikant's updated solution design document and sign off if it is acceptable.</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>Ayush</t>
         </is>
       </c>
-      <c r="C14" s="16" t="inlineStr">
+      <c r="C14" s="17" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D14" s="16" t="inlineStr">
+      <c r="D14" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E14" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="F14" s="15" t="inlineStr">
+      <c r="E14" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G14" s="15" t="inlineStr">
+      <c r="G14" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H14" s="15" t="inlineStr"/>
-      <c r="I14" s="15" t="inlineStr"/>
-      <c r="J14" s="15" t="inlineStr"/>
-      <c r="K14" s="16" t="inlineStr"/>
-      <c r="L14" s="15" t="inlineStr"/>
-      <c r="M14" s="15" t="inlineStr"/>
-      <c r="N14" s="15" t="inlineStr"/>
-      <c r="O14" s="15" t="inlineStr">
+      <c r="H14" s="16" t="inlineStr"/>
+      <c r="I14" s="16" t="inlineStr"/>
+      <c r="J14" s="16" t="inlineStr"/>
+      <c r="K14" s="17" t="inlineStr"/>
+      <c r="L14" s="16" t="inlineStr"/>
+      <c r="M14" s="16" t="inlineStr"/>
+      <c r="N14" s="16" t="inlineStr"/>
+      <c r="O14" s="16" t="inlineStr">
         <is>
           <t>He sent it to me. I'll review it and I'll sign off on that if it is okay.</t>
         </is>
       </c>
-      <c r="P14" s="15" t="inlineStr"/>
-      <c r="Q14" s="15" t="inlineStr">
+      <c r="P14" s="16" t="inlineStr"/>
+      <c r="Q14" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R14" s="16" t="inlineStr">
+      <c r="R14" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S14" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T14" s="17" t="n"/>
-      <c r="U14" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="V14" s="15" t="inlineStr">
+      <c r="S14" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T14" s="18" t="n"/>
+      <c r="U14" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="V14" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W14" s="15" t="inlineStr">
+      <c r="W14" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-intelligent-tracker-07</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Show Sreekumar in the application how CR items and issues resolve into work-item tasks.</t>
         </is>
       </c>
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>Ashwini</t>
         </is>
       </c>
-      <c r="C15" s="16" t="inlineStr">
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E15" s="17" t="n"/>
-      <c r="F15" s="15" t="inlineStr">
+      <c r="E15" s="18" t="n"/>
+      <c r="F15" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G15" s="15" t="inlineStr">
+      <c r="G15" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H15" s="15" t="inlineStr"/>
-      <c r="I15" s="15" t="inlineStr"/>
-      <c r="J15" s="15" t="inlineStr"/>
-      <c r="K15" s="16" t="inlineStr"/>
-      <c r="L15" s="15" t="inlineStr"/>
-      <c r="M15" s="15" t="inlineStr"/>
-      <c r="N15" s="15" t="inlineStr"/>
-      <c r="O15" s="15" t="inlineStr">
+      <c r="H15" s="16" t="inlineStr"/>
+      <c r="I15" s="16" t="inlineStr"/>
+      <c r="J15" s="16" t="inlineStr"/>
+      <c r="K15" s="17" t="inlineStr"/>
+      <c r="L15" s="16" t="inlineStr"/>
+      <c r="M15" s="16" t="inlineStr"/>
+      <c r="N15" s="16" t="inlineStr"/>
+      <c r="O15" s="16" t="inlineStr">
         <is>
           <t>Yeah, that we will show you on the website.</t>
         </is>
       </c>
-      <c r="P15" s="15" t="inlineStr"/>
-      <c r="Q15" s="15" t="inlineStr">
+      <c r="P15" s="16" t="inlineStr"/>
+      <c r="Q15" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R15" s="16" t="inlineStr">
+      <c r="R15" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S15" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T15" s="17" t="n"/>
-      <c r="U15" s="17" t="n">
+      <c r="S15" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T15" s="18" t="n"/>
+      <c r="U15" s="18" t="n">
         <v>46280</v>
       </c>
-      <c r="V15" s="15" t="inlineStr">
+      <c r="V15" s="16" t="inlineStr">
         <is>
           <t>2026-09-15-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W15" s="15" t="inlineStr">
+      <c r="W15" s="16" t="inlineStr">
         <is>
           <t>2026-09-15-intelligent-tracker-03</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Log detailed CR module tasks for today in Zoho and send the task ID to Ashwini.</t>
         </is>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>Johan</t>
         </is>
       </c>
-      <c r="C16" s="16" t="inlineStr">
+      <c r="C16" s="17" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr">
+      <c r="D16" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E16" s="17" t="n">
+      <c r="E16" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="F16" s="15" t="inlineStr">
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G16" s="15" t="inlineStr">
+      <c r="G16" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H16" s="15" t="inlineStr"/>
-      <c r="I16" s="15" t="inlineStr"/>
-      <c r="J16" s="15" t="inlineStr"/>
-      <c r="K16" s="16" t="inlineStr"/>
-      <c r="L16" s="15" t="inlineStr"/>
-      <c r="M16" s="15" t="inlineStr"/>
-      <c r="N16" s="15" t="inlineStr"/>
-      <c r="O16" s="15" t="inlineStr">
+      <c r="H16" s="16" t="inlineStr"/>
+      <c r="I16" s="16" t="inlineStr"/>
+      <c r="J16" s="16" t="inlineStr"/>
+      <c r="K16" s="17" t="inlineStr"/>
+      <c r="L16" s="16" t="inlineStr"/>
+      <c r="M16" s="16" t="inlineStr"/>
+      <c r="N16" s="16" t="inlineStr"/>
+      <c r="O16" s="16" t="inlineStr">
         <is>
           <t>they will be noting down their detailed task in Zoho and giving a Task ID to Ashwini</t>
         </is>
       </c>
-      <c r="P16" s="15" t="inlineStr"/>
-      <c r="Q16" s="15" t="inlineStr">
+      <c r="P16" s="16" t="inlineStr"/>
+      <c r="Q16" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R16" s="16" t="inlineStr">
+      <c r="R16" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S16" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T16" s="17" t="n"/>
-      <c r="U16" s="17" t="n">
+      <c r="S16" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T16" s="18" t="n"/>
+      <c r="U16" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="V16" s="15" t="inlineStr">
+      <c r="V16" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W16" s="15" t="inlineStr">
+      <c r="W16" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-intelligent-tracker-02</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Log detailed Issues module tasks for today in Zoho and send the task ID to Ashwini.</t>
         </is>
       </c>
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr">
         <is>
           <t>Samuel</t>
         </is>
       </c>
-      <c r="C17" s="16" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E17" s="17" t="n">
+      <c r="E17" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="F17" s="15" t="inlineStr">
+      <c r="F17" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G17" s="15" t="inlineStr">
+      <c r="G17" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H17" s="15" t="inlineStr"/>
-      <c r="I17" s="15" t="inlineStr"/>
-      <c r="J17" s="15" t="inlineStr"/>
-      <c r="K17" s="16" t="inlineStr"/>
-      <c r="L17" s="15" t="inlineStr"/>
-      <c r="M17" s="15" t="inlineStr"/>
-      <c r="N17" s="15" t="inlineStr"/>
-      <c r="O17" s="15" t="inlineStr">
+      <c r="H17" s="16" t="inlineStr"/>
+      <c r="I17" s="16" t="inlineStr"/>
+      <c r="J17" s="16" t="inlineStr"/>
+      <c r="K17" s="17" t="inlineStr"/>
+      <c r="L17" s="16" t="inlineStr"/>
+      <c r="M17" s="16" t="inlineStr"/>
+      <c r="N17" s="16" t="inlineStr"/>
+      <c r="O17" s="16" t="inlineStr">
         <is>
           <t>they will be noting down their detailed task in Zoho and giving a Task ID to Ashwini</t>
         </is>
       </c>
-      <c r="P17" s="15" t="inlineStr"/>
-      <c r="Q17" s="15" t="inlineStr">
+      <c r="P17" s="16" t="inlineStr"/>
+      <c r="Q17" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R17" s="16" t="inlineStr">
+      <c r="R17" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S17" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T17" s="17" t="n"/>
-      <c r="U17" s="17" t="n">
+      <c r="S17" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T17" s="18" t="n"/>
+      <c r="U17" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="V17" s="15" t="inlineStr">
+      <c r="V17" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W17" s="15" t="inlineStr">
+      <c r="W17" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-intelligent-tracker-03</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>Speak with Laxmikant to plan the development plan and model for the build.</t>
         </is>
       </c>
-      <c r="B18" s="15" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
         <is>
           <t>Ayush</t>
         </is>
       </c>
-      <c r="C18" s="16" t="inlineStr">
+      <c r="C18" s="17" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D18" s="16" t="inlineStr">
+      <c r="D18" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E18" s="17" t="n">
+      <c r="E18" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="F18" s="15" t="inlineStr">
+      <c r="F18" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G18" s="15" t="inlineStr">
+      <c r="G18" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H18" s="15" t="inlineStr"/>
-      <c r="I18" s="15" t="inlineStr"/>
-      <c r="J18" s="15" t="inlineStr"/>
-      <c r="K18" s="16" t="inlineStr"/>
-      <c r="L18" s="15" t="inlineStr"/>
-      <c r="M18" s="15" t="inlineStr"/>
-      <c r="N18" s="15" t="inlineStr"/>
-      <c r="O18" s="15" t="inlineStr">
+      <c r="H18" s="16" t="inlineStr"/>
+      <c r="I18" s="16" t="inlineStr"/>
+      <c r="J18" s="16" t="inlineStr"/>
+      <c r="K18" s="17" t="inlineStr"/>
+      <c r="L18" s="16" t="inlineStr"/>
+      <c r="M18" s="16" t="inlineStr"/>
+      <c r="N18" s="16" t="inlineStr"/>
+      <c r="O18" s="16" t="inlineStr">
         <is>
           <t>I will speak to Lakshmi, plan development plan with model that's it</t>
         </is>
       </c>
-      <c r="P18" s="15" t="inlineStr"/>
-      <c r="Q18" s="15" t="inlineStr">
+      <c r="P18" s="16" t="inlineStr"/>
+      <c r="Q18" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R18" s="16" t="inlineStr">
+      <c r="R18" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S18" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T18" s="17" t="n"/>
-      <c r="U18" s="17" t="n">
+      <c r="S18" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T18" s="18" t="n"/>
+      <c r="U18" s="18" t="n">
         <v>46276</v>
       </c>
-      <c r="V18" s="15" t="inlineStr">
+      <c r="V18" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W18" s="15" t="inlineStr">
+      <c r="W18" s="16" t="inlineStr">
         <is>
           <t>2026-09-11-intelligent-tracker-08</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>Discuss with Laxmikant the feasibility and structural changes needed for the new issue fields from Sreekumar's design before building them.</t>
         </is>
       </c>
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>Samuel</t>
         </is>
       </c>
-      <c r="C19" s="16" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="D19" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E19" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="F19" s="15" t="inlineStr">
+      <c r="E19" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
         <is>
           <t>intelligent-tracker</t>
         </is>
       </c>
-      <c r="G19" s="15" t="inlineStr">
+      <c r="G19" s="16" t="inlineStr">
         <is>
           <t>Intelligent Tracker</t>
         </is>
       </c>
-      <c r="H19" s="15" t="inlineStr"/>
-      <c r="I19" s="15" t="inlineStr"/>
-      <c r="J19" s="15" t="inlineStr"/>
-      <c r="K19" s="16" t="inlineStr"/>
-      <c r="L19" s="15" t="inlineStr"/>
-      <c r="M19" s="15" t="inlineStr"/>
-      <c r="N19" s="15" t="inlineStr"/>
-      <c r="O19" s="15" t="inlineStr">
+      <c r="H19" s="16" t="inlineStr"/>
+      <c r="I19" s="16" t="inlineStr"/>
+      <c r="J19" s="16" t="inlineStr"/>
+      <c r="K19" s="17" t="inlineStr"/>
+      <c r="L19" s="16" t="inlineStr"/>
+      <c r="M19" s="16" t="inlineStr"/>
+      <c r="N19" s="16" t="inlineStr"/>
+      <c r="O19" s="16" t="inlineStr">
         <is>
           <t>I wanted Sam to talk to you regarding the feasibility of that. I know it will work, but what is the structure change?</t>
         </is>
       </c>
-      <c r="P19" s="15" t="inlineStr"/>
-      <c r="Q19" s="15" t="inlineStr">
+      <c r="P19" s="16" t="inlineStr"/>
+      <c r="Q19" s="16" t="inlineStr">
         <is>
           <t>Activity Tracker internal sync-up</t>
         </is>
       </c>
-      <c r="R19" s="16" t="inlineStr">
+      <c r="R19" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S19" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T19" s="17" t="n"/>
-      <c r="U19" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="V19" s="15" t="inlineStr">
+      <c r="S19" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T19" s="18" t="n"/>
+      <c r="U19" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="V19" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-activity-tracker-sync.md</t>
         </is>
       </c>
-      <c r="W19" s="15" t="inlineStr">
+      <c r="W19" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-intelligent-tracker-01</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>Send out a skill-gap poll on HTML/CSS/JavaScript proficiency and use the results to build the training plan.</t>
         </is>
       </c>
-      <c r="B20" s="15" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
         <is>
           <t>Sarathchandra Babu</t>
         </is>
       </c>
-      <c r="C20" s="16" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D20" s="16" t="inlineStr">
+      <c r="D20" s="17" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="E20" s="17" t="n">
+      <c r="E20" s="18" t="n">
         <v>46282</v>
       </c>
-      <c r="F20" s="15" t="inlineStr">
+      <c r="F20" s="16" t="inlineStr">
         <is>
           <t>unassigned</t>
         </is>
       </c>
-      <c r="G20" s="15" t="inlineStr">
+      <c r="G20" s="16" t="inlineStr">
         <is>
           <t>unassigned</t>
         </is>
       </c>
-      <c r="H20" s="15" t="inlineStr">
+      <c r="H20" s="16" t="inlineStr">
         <is>
           <t>coordinate</t>
         </is>
       </c>
-      <c r="I20" s="15" t="inlineStr">
+      <c r="I20" s="16" t="inlineStr">
         <is>
           <t>Send the poll to the team and collect responses.</t>
         </is>
       </c>
-      <c r="J20" s="15" t="inlineStr"/>
-      <c r="K20" s="16" t="inlineStr">
+      <c r="J20" s="16" t="inlineStr"/>
+      <c r="K20" s="17" t="inlineStr">
         <is>
           <t>1h</t>
         </is>
       </c>
-      <c r="L20" s="15" t="inlineStr"/>
-      <c r="M20" s="15" t="inlineStr"/>
-      <c r="N20" s="15" t="inlineStr"/>
-      <c r="O20" s="15" t="inlineStr">
+      <c r="L20" s="16" t="inlineStr"/>
+      <c r="M20" s="16" t="inlineStr"/>
+      <c r="N20" s="16" t="inlineStr"/>
+      <c r="O20" s="16" t="inlineStr">
         <is>
           <t>Or, if you can put a poll in one of these, let's see here.</t>
         </is>
       </c>
-      <c r="P20" s="15" t="inlineStr">
+      <c r="P20" s="16" t="inlineStr">
         <is>
           <t>D-2026-09-17-02</t>
         </is>
       </c>
-      <c r="Q20" s="15" t="inlineStr">
+      <c r="Q20" s="16" t="inlineStr">
         <is>
           <t>Code Apps Learning Curriculum Structure Discussion</t>
         </is>
       </c>
-      <c r="R20" s="16" t="inlineStr">
+      <c r="R20" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S20" s="17" t="n">
+      <c r="S20" s="18" t="n">
         <v>46282</v>
       </c>
-      <c r="T20" s="17" t="n"/>
-      <c r="U20" s="17" t="n">
+      <c r="T20" s="18" t="n"/>
+      <c r="U20" s="18" t="n">
         <v>46282</v>
       </c>
-      <c r="V20" s="15" t="inlineStr">
+      <c r="V20" s="16" t="inlineStr">
         <is>
           <t>2026-09-17-code-apps-learning-curriculum-discussion.docx</t>
         </is>
       </c>
-      <c r="W20" s="15" t="inlineStr">
+      <c r="W20" s="16" t="inlineStr">
         <is>
           <t>2026-09-17-unassigned-01</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>Review the new lsp_claim_line_items table and added claim-table columns against the no-further-master-data-changes position agreed with Adwaith.</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>Ayush</t>
         </is>
       </c>
-      <c r="C21" s="16" t="inlineStr">
+      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D21" s="16" t="inlineStr">
+      <c r="D21" s="17" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="E21" s="17" t="n"/>
-      <c r="F21" s="15" t="inlineStr">
+      <c r="E21" s="18" t="n"/>
+      <c r="F21" s="16" t="inlineStr">
         <is>
           <t>lsp</t>
         </is>
       </c>
-      <c r="G21" s="15" t="inlineStr">
+      <c r="G21" s="16" t="inlineStr">
         <is>
           <t>unassigned</t>
         </is>
       </c>
-      <c r="H21" s="15" t="inlineStr">
+      <c r="H21" s="16" t="inlineStr">
         <is>
           <t>review</t>
         </is>
       </c>
-      <c r="I21" s="15" t="inlineStr">
+      <c r="I21" s="16" t="inlineStr">
         <is>
           <t>Ayush compares the new tables and columns against the sign-off position and flags any conflicts to Adwaith.</t>
         </is>
       </c>
-      <c r="J21" s="15" t="inlineStr"/>
-      <c r="K21" s="16" t="inlineStr">
+      <c r="J21" s="16" t="inlineStr"/>
+      <c r="K21" s="17" t="inlineStr">
         <is>
           <t>half-day</t>
         </is>
       </c>
-      <c r="L21" s="15" t="inlineStr"/>
-      <c r="M21" s="15" t="inlineStr">
+      <c r="L21" s="16" t="inlineStr"/>
+      <c r="M21" s="16" t="inlineStr">
         <is>
           <t>List of new columns/tables from this CR</t>
         </is>
       </c>
-      <c r="N21" s="15" t="inlineStr"/>
-      <c r="O21" s="15" t="inlineStr">
+      <c r="N21" s="16" t="inlineStr"/>
+      <c r="O21" s="16" t="inlineStr">
         <is>
           <t>Existing claim table: add lsp_fy, lsp_totalnrclaimwithsr, lsp_totalpoclaimwithsr, plus the status-sync fields</t>
         </is>
       </c>
-      <c r="P21" s="15" t="inlineStr">
+      <c r="P21" s="16" t="inlineStr">
         <is>
           <t>No further master data or DB column changes after sign-off (told to Adwaith on 2026-09-16).</t>
         </is>
       </c>
-      <c r="Q21" s="15" t="inlineStr">
+      <c r="Q21" s="16" t="inlineStr">
         <is>
           <t>CR: Distributor Line-Item Visibility and Claim Status Sync</t>
         </is>
       </c>
-      <c r="R21" s="16" t="inlineStr">
+      <c r="R21" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S21" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T21" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="U21" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="V21" s="15" t="inlineStr">
+      <c r="S21" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T21" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="U21" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="V21" s="16" t="inlineStr">
         <is>
           <t>CR_DISTRIBUTOR_LINE_ITEM_VISIBILITY_Revised (1).docx</t>
         </is>
       </c>
-      <c r="W21" s="15" t="inlineStr">
+      <c r="W21" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-lsp-01</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>Populate lsp_distributoremail for every distributor before the claim-status notification feature rolls out.</t>
         </is>
       </c>
-      <c r="B22" s="15" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>Adwaith</t>
         </is>
       </c>
-      <c r="C22" s="16" t="inlineStr">
+      <c r="C22" s="17" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D22" s="16" t="inlineStr">
+      <c r="D22" s="17" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="E22" s="17" t="n"/>
-      <c r="F22" s="15" t="inlineStr">
+      <c r="E22" s="18" t="n"/>
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>lsp</t>
         </is>
       </c>
-      <c r="G22" s="15" t="inlineStr">
+      <c r="G22" s="16" t="inlineStr">
         <is>
           <t>unassigned</t>
         </is>
       </c>
-      <c r="H22" s="15" t="inlineStr">
+      <c r="H22" s="16" t="inlineStr">
         <is>
           <t>other</t>
         </is>
       </c>
-      <c r="I22" s="15" t="inlineStr">
+      <c r="I22" s="16" t="inlineStr">
         <is>
           <t>Adwaith supplies the missing distributor email addresses for all distributor master records.</t>
         </is>
       </c>
-      <c r="J22" s="15" t="inlineStr"/>
-      <c r="K22" s="16" t="inlineStr">
+      <c r="J22" s="16" t="inlineStr"/>
+      <c r="K22" s="17" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="L22" s="15" t="inlineStr"/>
-      <c r="M22" s="15" t="inlineStr"/>
-      <c r="N22" s="15" t="inlineStr"/>
-      <c r="O22" s="15" t="inlineStr">
+      <c r="L22" s="16" t="inlineStr"/>
+      <c r="M22" s="16" t="inlineStr"/>
+      <c r="N22" s="16" t="inlineStr"/>
+      <c r="O22" s="16" t="inlineStr">
         <is>
           <t>lsp_distributoremail is not populated for every distributor. Populate it before rollout or the notification silently sends to nobody.</t>
         </is>
       </c>
-      <c r="P22" s="15" t="inlineStr">
+      <c r="P22" s="16" t="inlineStr">
         <is>
           <t>CR section 7.4 Notifications</t>
         </is>
       </c>
-      <c r="Q22" s="15" t="inlineStr">
+      <c r="Q22" s="16" t="inlineStr">
         <is>
           <t>CR: Distributor Line-Item Visibility and Claim Status Sync</t>
         </is>
       </c>
-      <c r="R22" s="16" t="inlineStr">
+      <c r="R22" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S22" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T22" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="U22" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="V22" s="15" t="inlineStr">
+      <c r="S22" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T22" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="U22" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="V22" s="16" t="inlineStr">
         <is>
           <t>CR_DISTRIBUTOR_LINE_ITEM_VISIBILITY_Revised (1).docx</t>
         </is>
       </c>
-      <c r="W22" s="15" t="inlineStr">
+      <c r="W22" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-lsp-02</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>Agree and document a retention or archival policy for closed periodic closure line-item data.</t>
         </is>
       </c>
-      <c r="B23" s="15" t="inlineStr">
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>Ayush</t>
         </is>
       </c>
-      <c r="C23" s="16" t="inlineStr">
+      <c r="C23" s="17" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="D23" s="16" t="inlineStr">
+      <c r="D23" s="17" t="inlineStr">
         <is>
           <t>done</t>
         </is>
       </c>
-      <c r="E23" s="17" t="n"/>
-      <c r="F23" s="15" t="inlineStr">
+      <c r="E23" s="18" t="n"/>
+      <c r="F23" s="16" t="inlineStr">
         <is>
           <t>lsp</t>
         </is>
       </c>
-      <c r="G23" s="15" t="inlineStr">
+      <c r="G23" s="16" t="inlineStr">
         <is>
           <t>unassigned</t>
         </is>
       </c>
-      <c r="H23" s="15" t="inlineStr">
+      <c r="H23" s="16" t="inlineStr">
         <is>
           <t>decide</t>
         </is>
       </c>
-      <c r="I23" s="15" t="inlineStr">
+      <c r="I23" s="16" t="inlineStr">
         <is>
           <t>Ayush proposes a retention window and confirms it with the DMS side.</t>
         </is>
       </c>
-      <c r="J23" s="15" t="inlineStr"/>
-      <c r="K23" s="16" t="inlineStr">
+      <c r="J23" s="16" t="inlineStr"/>
+      <c r="K23" s="17" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="L23" s="15" t="inlineStr"/>
-      <c r="M23" s="15" t="inlineStr"/>
-      <c r="N23" s="15" t="inlineStr"/>
-      <c r="O23" s="15" t="inlineStr">
+      <c r="L23" s="16" t="inlineStr"/>
+      <c r="M23" s="16" t="inlineStr"/>
+      <c r="N23" s="16" t="inlineStr"/>
+      <c r="O23" s="16" t="inlineStr">
         <is>
           <t>Agree a retention or archival policy for closed periodic closures.</t>
         </is>
       </c>
-      <c r="P23" s="15" t="inlineStr">
+      <c r="P23" s="16" t="inlineStr">
         <is>
           <t>CR section 8.6 Sizing</t>
         </is>
       </c>
-      <c r="Q23" s="15" t="inlineStr">
+      <c r="Q23" s="16" t="inlineStr">
         <is>
           <t>CR: Distributor Line-Item Visibility and Claim Status Sync</t>
         </is>
       </c>
-      <c r="R23" s="16" t="inlineStr">
+      <c r="R23" s="17" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="S23" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="T23" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="U23" s="17" t="n">
-        <v>46281</v>
-      </c>
-      <c r="V23" s="15" t="inlineStr">
+      <c r="S23" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="T23" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="U23" s="18" t="n">
+        <v>46281</v>
+      </c>
+      <c r="V23" s="16" t="inlineStr">
         <is>
           <t>CR_DISTRIBUTOR_LINE_ITEM_VISIBILITY_Revised (1).docx</t>
         </is>
       </c>
-      <c r="W23" s="15" t="inlineStr">
+      <c r="W23" s="16" t="inlineStr">
         <is>
           <t>2026-09-16-lsp-03</t>
         </is>
@@ -3449,40 +3534,40 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D5000">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="1" dxfId="1">
       <formula>$D2="done"</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
+    <cfRule type="expression" priority="2" dxfId="2">
       <formula>$D2="to_verify"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="2">
+    <cfRule type="expression" priority="3" dxfId="3">
       <formula>$D2="blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="3">
+    <cfRule type="expression" priority="4" dxfId="4">
       <formula>$D2="in_progress"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C5000">
-    <cfRule type="expression" priority="5" dxfId="4">
+    <cfRule type="expression" priority="5" dxfId="5">
       <formula>AND($C2="P1",NOT(OR($D2="done",$D2="rejected")))</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="5">
+    <cfRule type="expression" priority="6" dxfId="6">
       <formula>AND($C2="P2",NOT(OR($D2="done",$D2="rejected")))</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" dxfId="6">
+    <cfRule type="expression" priority="7" dxfId="7">
       <formula>AND($C2="P3",NOT(OR($D2="done",$D2="rejected")))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E5000">
-    <cfRule type="expression" priority="8" dxfId="7">
+    <cfRule type="expression" priority="8" dxfId="8">
       <formula>AND($E2&lt;&gt;"",$E2&lt;TODAY(),NOT(OR($D2="done",$D2="rejected")))</formula>
     </cfRule>
-    <cfRule type="expression" priority="9" dxfId="8">
+    <cfRule type="expression" priority="9" dxfId="9">
       <formula>AND($E2&lt;&gt;"",$E2=TODAY(),NOT(OR($D2="done",$D2="rejected")))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:W5000">
-    <cfRule type="expression" priority="10" dxfId="9">
+    <cfRule type="expression" priority="10" dxfId="10">
       <formula>OR($D2="done",$D2="rejected")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>